<commit_message>
Actualizacion automatica de siprem_latest.xlsx
</commit_message>
<xml_diff>
--- a/siprem_latest.xlsx
+++ b/siprem_latest.xlsx
@@ -29,7 +29,7 @@
     <t>FECHA</t>
   </si>
   <si>
-    <t>18/07/2026 a las 07:25:17</t>
+    <t>18/07/2026 a las 07:39:02</t>
   </si>
   <si>
     <t>Num_Lote</t>
@@ -6182,7 +6182,7 @@
         <v>1</v>
       </c>
       <c r="X27" s="4" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="Y27" s="4"/>
       <c r="Z27" s="4" t="s">
@@ -11332,7 +11332,7 @@
         <v>3</v>
       </c>
       <c r="X95" s="4" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="Y95" s="4"/>
       <c r="Z95" s="4" t="s">
@@ -21320,7 +21320,7 @@
         <v>2</v>
       </c>
       <c r="X227" s="4" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="Y227" s="4"/>
       <c r="Z227" s="4" t="s">
@@ -23264,7 +23264,7 @@
         <v>2</v>
       </c>
       <c r="X254" s="4" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="Y254" s="4"/>
       <c r="Z254" s="4" t="s">
@@ -23416,7 +23416,7 @@
         <v>1</v>
       </c>
       <c r="X256" s="4" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="Y256" s="4"/>
       <c r="Z256" s="4" t="s">
@@ -24762,7 +24762,7 @@
         <v>1</v>
       </c>
       <c r="X274" s="4" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="Y274" s="4"/>
       <c r="Z274" s="4" t="s">
@@ -25260,7 +25260,7 @@
         <v>1</v>
       </c>
       <c r="X281" s="4" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="Y281" s="4"/>
       <c r="Z281" s="4" t="s">

</xml_diff>

<commit_message>
Actualizacion automatica SIPREM y Casuistica
</commit_message>
<xml_diff>
--- a/siprem_latest.xlsx
+++ b/siprem_latest.xlsx
@@ -29,7 +29,7 @@
     <t>FECHA</t>
   </si>
   <si>
-    <t>11/08/2026 a las 07:54:25</t>
+    <t>11/08/2026 a las 08:01:14</t>
   </si>
   <si>
     <t>Num_Lote</t>
@@ -17779,7 +17779,7 @@
         <v>5</v>
       </c>
       <c r="X171" s="4" t="s">
-        <v>543</v>
+        <v>148</v>
       </c>
       <c r="Y171" s="4"/>
       <c r="Z171" s="4" t="s">
@@ -20537,7 +20537,7 @@
         <v>8</v>
       </c>
       <c r="X207" s="4" t="s">
-        <v>543</v>
+        <v>148</v>
       </c>
       <c r="Y207" s="4"/>
       <c r="Z207" s="4" t="s">
@@ -25495,7 +25495,7 @@
         <v>7</v>
       </c>
       <c r="X272" s="4" t="s">
-        <v>543</v>
+        <v>148</v>
       </c>
       <c r="Y272" s="4"/>
       <c r="Z272" s="4" t="s">
@@ -28615,7 +28615,7 @@
         <v>7</v>
       </c>
       <c r="X316" s="4" t="s">
-        <v>543</v>
+        <v>148</v>
       </c>
       <c r="Y316" s="4"/>
       <c r="Z316" s="4" t="s">

</xml_diff>